<commit_message>
feat: add skill gap analysis workflow
</commit_message>
<xml_diff>
--- a/backend/models/excel/role_recommendation.xlsx
+++ b/backend/models/excel/role_recommendation.xlsx
@@ -1,18 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="22730"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Hasnain Raza\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1619A891-544B-4F1A-8C22-08D13CB18542}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7500"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Computing Professionals" sheetId="1" r:id="rId1"/>
+    <sheet name="Role Recommendation" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
@@ -504,7 +505,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -837,14 +838,14 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K501"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="10" max="10" width="22.7109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="22.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -879,7 +880,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>11</v>
       </c>
@@ -902,7 +903,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>18</v>
       </c>
@@ -934,7 +935,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>28</v>
       </c>
@@ -963,7 +964,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>36</v>
       </c>
@@ -992,7 +993,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>45</v>
       </c>
@@ -1021,7 +1022,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>19</v>
       </c>
@@ -1044,7 +1045,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>60</v>
       </c>
@@ -1073,7 +1074,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>68</v>
       </c>
@@ -1108,7 +1109,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>73</v>
       </c>
@@ -1131,7 +1132,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>78</v>
       </c>
@@ -1160,7 +1161,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>81</v>
       </c>
@@ -1180,7 +1181,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>19</v>
       </c>
@@ -1212,7 +1213,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>87</v>
       </c>
@@ -1247,7 +1248,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>96</v>
       </c>
@@ -1279,7 +1280,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>105</v>
       </c>
@@ -1308,7 +1309,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>109</v>
       </c>
@@ -1340,7 +1341,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>29</v>
       </c>
@@ -1360,7 +1361,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>62</v>
       </c>
@@ -1395,7 +1396,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>49</v>
       </c>
@@ -1427,7 +1428,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>41</v>
       </c>
@@ -1462,7 +1463,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>28</v>
       </c>
@@ -1494,7 +1495,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>11</v>
       </c>
@@ -1523,7 +1524,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>110</v>
       </c>
@@ -1549,7 +1550,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>123</v>
       </c>
@@ -1578,7 +1579,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>70</v>
       </c>
@@ -1604,7 +1605,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>114</v>
       </c>
@@ -1636,7 +1637,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>13</v>
       </c>
@@ -1659,7 +1660,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>46</v>
       </c>
@@ -1679,7 +1680,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>127</v>
       </c>
@@ -1711,7 +1712,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>84</v>
       </c>
@@ -1743,7 +1744,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>41</v>
       </c>
@@ -1769,7 +1770,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>134</v>
       </c>
@@ -1798,7 +1799,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>57</v>
       </c>
@@ -1833,7 +1834,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>76</v>
       </c>
@@ -1865,7 +1866,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>63</v>
       </c>
@@ -1897,7 +1898,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>49</v>
       </c>
@@ -1917,7 +1918,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>54</v>
       </c>
@@ -1952,7 +1953,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>30</v>
       </c>
@@ -1975,7 +1976,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>73</v>
       </c>
@@ -2010,7 +2011,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>84</v>
       </c>
@@ -2045,7 +2046,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>88</v>
       </c>
@@ -2077,7 +2078,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>46</v>
       </c>
@@ -2097,7 +2098,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>11</v>
       </c>
@@ -2132,7 +2133,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>13</v>
       </c>
@@ -2161,7 +2162,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>117</v>
       </c>
@@ -2196,7 +2197,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>122</v>
       </c>
@@ -2216,7 +2217,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>24</v>
       </c>
@@ -2248,7 +2249,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>47</v>
       </c>
@@ -2271,7 +2272,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>28</v>
       </c>
@@ -2291,7 +2292,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>70</v>
       </c>
@@ -2317,7 +2318,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>50</v>
       </c>
@@ -2346,7 +2347,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>112</v>
       </c>
@@ -2381,7 +2382,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>20</v>
       </c>
@@ -2407,7 +2408,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>57</v>
       </c>
@@ -2439,7 +2440,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>28</v>
       </c>
@@ -2462,7 +2463,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="57" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>39</v>
       </c>
@@ -2485,7 +2486,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="58" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>96</v>
       </c>
@@ -2511,7 +2512,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>79</v>
       </c>
@@ -2540,7 +2541,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="60" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>56</v>
       </c>
@@ -2560,7 +2561,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="61" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>88</v>
       </c>
@@ -2586,7 +2587,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>146</v>
       </c>
@@ -2615,7 +2616,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>107</v>
       </c>
@@ -2638,7 +2639,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="64" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>144</v>
       </c>
@@ -2670,7 +2671,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="65" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>79</v>
       </c>
@@ -2702,7 +2703,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="66" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
         <v>82</v>
       </c>
@@ -2737,7 +2738,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="67" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>105</v>
       </c>
@@ -2760,7 +2761,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="68" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
         <v>51</v>
       </c>
@@ -2786,7 +2787,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="69" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
         <v>47</v>
       </c>
@@ -2806,7 +2807,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="70" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
         <v>39</v>
       </c>
@@ -2841,7 +2842,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="71" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>28</v>
       </c>
@@ -2864,7 +2865,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="72" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
         <v>125</v>
       </c>
@@ -2896,7 +2897,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="73" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>71</v>
       </c>
@@ -2922,7 +2923,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="74" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
         <v>22</v>
       </c>
@@ -2945,7 +2946,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="75" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
         <v>89</v>
       </c>
@@ -2974,7 +2975,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="76" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
         <v>22</v>
       </c>
@@ -3003,7 +3004,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="77" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
         <v>14</v>
       </c>
@@ -3035,7 +3036,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="78" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
         <v>50</v>
       </c>
@@ -3067,7 +3068,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="79" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
         <v>150</v>
       </c>
@@ -3090,7 +3091,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="80" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
         <v>139</v>
       </c>
@@ -3125,7 +3126,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="81" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
         <v>28</v>
       </c>
@@ -3154,7 +3155,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="82" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
         <v>25</v>
       </c>
@@ -3189,7 +3190,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="83" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
         <v>11</v>
       </c>
@@ -3209,7 +3210,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="84" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
         <v>136</v>
       </c>
@@ -3229,7 +3230,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="85" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
         <v>107</v>
       </c>
@@ -3252,7 +3253,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="86" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
         <v>19</v>
       </c>
@@ -3284,7 +3285,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="87" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
         <v>30</v>
       </c>
@@ -3304,7 +3305,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="88" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
         <v>123</v>
       </c>
@@ -3336,7 +3337,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="89" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
         <v>68</v>
       </c>
@@ -3368,7 +3369,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="90" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
         <v>140</v>
       </c>
@@ -3391,7 +3392,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="91" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A91" t="s">
         <v>123</v>
       </c>
@@ -3420,7 +3421,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="92" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
         <v>21</v>
       </c>
@@ -3455,7 +3456,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="93" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
         <v>61</v>
       </c>
@@ -3484,7 +3485,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="94" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A94" t="s">
         <v>14</v>
       </c>
@@ -3519,7 +3520,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="95" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
         <v>100</v>
       </c>
@@ -3554,7 +3555,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="96" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A96" t="s">
         <v>12</v>
       </c>
@@ -3577,7 +3578,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="97" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A97" t="s">
         <v>33</v>
       </c>
@@ -3597,7 +3598,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="98" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A98" t="s">
         <v>137</v>
       </c>
@@ -3623,7 +3624,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="99" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A99" t="s">
         <v>54</v>
       </c>
@@ -3658,7 +3659,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="100" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A100" t="s">
         <v>90</v>
       </c>
@@ -3684,7 +3685,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="101" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A101" t="s">
         <v>13</v>
       </c>
@@ -3716,7 +3717,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="102" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A102" t="s">
         <v>123</v>
       </c>
@@ -3748,7 +3749,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="103" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A103" t="s">
         <v>46</v>
       </c>
@@ -3777,7 +3778,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="104" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A104" t="s">
         <v>43</v>
       </c>
@@ -3800,7 +3801,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="105" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A105" t="s">
         <v>28</v>
       </c>
@@ -3826,7 +3827,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="106" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A106" t="s">
         <v>61</v>
       </c>
@@ -3858,7 +3859,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="107" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A107" t="s">
         <v>88</v>
       </c>
@@ -3881,7 +3882,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="108" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A108" t="s">
         <v>39</v>
       </c>
@@ -3907,7 +3908,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="109" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A109" t="s">
         <v>51</v>
       </c>
@@ -3933,7 +3934,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="110" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A110" t="s">
         <v>75</v>
       </c>
@@ -3953,7 +3954,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="111" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A111" t="s">
         <v>98</v>
       </c>
@@ -3982,7 +3983,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="112" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A112" t="s">
         <v>20</v>
       </c>
@@ -4005,7 +4006,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="113" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A113" t="s">
         <v>147</v>
       </c>
@@ -4040,7 +4041,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="114" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A114" t="s">
         <v>56</v>
       </c>
@@ -4075,7 +4076,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="115" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A115" t="s">
         <v>28</v>
       </c>
@@ -4107,7 +4108,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="116" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A116" t="s">
         <v>76</v>
       </c>
@@ -4136,7 +4137,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="117" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A117" t="s">
         <v>36</v>
       </c>
@@ -4171,7 +4172,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="118" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A118" t="s">
         <v>86</v>
       </c>
@@ -4197,7 +4198,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="119" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A119" t="s">
         <v>154</v>
       </c>
@@ -4226,7 +4227,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="120" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A120" t="s">
         <v>68</v>
       </c>
@@ -4255,7 +4256,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="121" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A121" t="s">
         <v>100</v>
       </c>
@@ -4287,7 +4288,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="122" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A122" t="s">
         <v>65</v>
       </c>
@@ -4307,7 +4308,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="123" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A123" t="s">
         <v>36</v>
       </c>
@@ -4336,7 +4337,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="124" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A124" t="s">
         <v>30</v>
       </c>
@@ -4368,7 +4369,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="125" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A125" t="s">
         <v>84</v>
       </c>
@@ -4394,7 +4395,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="126" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A126" t="s">
         <v>13</v>
       </c>
@@ -4426,7 +4427,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="127" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A127" t="s">
         <v>30</v>
       </c>
@@ -4449,7 +4450,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="128" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A128" t="s">
         <v>121</v>
       </c>
@@ -4481,7 +4482,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="129" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A129" t="s">
         <v>12</v>
       </c>
@@ -4507,7 +4508,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="130" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A130" t="s">
         <v>19</v>
       </c>
@@ -4539,7 +4540,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="131" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A131" t="s">
         <v>36</v>
       </c>
@@ -4565,7 +4566,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="132" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A132" t="s">
         <v>22</v>
       </c>
@@ -4600,7 +4601,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="133" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A133" t="s">
         <v>54</v>
       </c>
@@ -4632,7 +4633,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="134" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A134" t="s">
         <v>14</v>
       </c>
@@ -4652,7 +4653,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="135" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A135" t="s">
         <v>29</v>
       </c>
@@ -4672,7 +4673,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="136" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A136" t="s">
         <v>76</v>
       </c>
@@ -4704,7 +4705,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="137" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A137" t="s">
         <v>68</v>
       </c>
@@ -4724,7 +4725,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="138" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A138" t="s">
         <v>147</v>
       </c>
@@ -4744,7 +4745,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="139" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A139" t="s">
         <v>12</v>
       </c>
@@ -4770,7 +4771,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="140" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A140" t="s">
         <v>13</v>
       </c>
@@ -4802,7 +4803,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="141" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A141" t="s">
         <v>12</v>
       </c>
@@ -4831,7 +4832,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="142" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A142" t="s">
         <v>142</v>
       </c>
@@ -4857,7 +4858,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="143" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A143" t="s">
         <v>139</v>
       </c>
@@ -4892,7 +4893,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="144" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A144" t="s">
         <v>89</v>
       </c>
@@ -4912,7 +4913,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="145" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A145" t="s">
         <v>28</v>
       </c>
@@ -4932,7 +4933,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="146" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A146" t="s">
         <v>28</v>
       </c>
@@ -4967,7 +4968,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="147" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A147" t="s">
         <v>49</v>
       </c>
@@ -4993,7 +4994,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="148" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A148" t="s">
         <v>118</v>
       </c>
@@ -5016,7 +5017,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="149" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A149" t="s">
         <v>19</v>
       </c>
@@ -5048,7 +5049,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="150" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A150" t="s">
         <v>118</v>
       </c>
@@ -5074,7 +5075,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="151" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A151" t="s">
         <v>120</v>
       </c>
@@ -5094,7 +5095,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="152" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A152" t="s">
         <v>13</v>
       </c>
@@ -5123,7 +5124,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="153" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A153" t="s">
         <v>70</v>
       </c>
@@ -5152,7 +5153,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="154" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A154" t="s">
         <v>13</v>
       </c>
@@ -5175,7 +5176,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="155" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A155" t="s">
         <v>21</v>
       </c>
@@ -5198,7 +5199,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="156" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A156" t="s">
         <v>138</v>
       </c>
@@ -5221,7 +5222,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="157" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A157" t="s">
         <v>120</v>
       </c>
@@ -5244,7 +5245,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="158" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A158" t="s">
         <v>22</v>
       </c>
@@ -5264,7 +5265,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="159" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A159" t="s">
         <v>92</v>
       </c>
@@ -5284,7 +5285,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="160" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A160" t="s">
         <v>84</v>
       </c>
@@ -5310,7 +5311,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="161" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A161" t="s">
         <v>132</v>
       </c>
@@ -5336,7 +5337,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="162" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A162" t="s">
         <v>43</v>
       </c>
@@ -5371,7 +5372,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="163" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A163" t="s">
         <v>28</v>
       </c>
@@ -5397,7 +5398,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="164" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A164" t="s">
         <v>154</v>
       </c>
@@ -5420,7 +5421,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="165" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A165" t="s">
         <v>94</v>
       </c>
@@ -5449,7 +5450,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="166" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A166" t="s">
         <v>100</v>
       </c>
@@ -5475,7 +5476,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="167" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A167" t="s">
         <v>124</v>
       </c>
@@ -5498,7 +5499,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="168" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A168" t="s">
         <v>66</v>
       </c>
@@ -5530,7 +5531,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="169" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A169" t="s">
         <v>118</v>
       </c>
@@ -5559,7 +5560,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="170" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A170" t="s">
         <v>60</v>
       </c>
@@ -5585,7 +5586,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="171" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A171" t="s">
         <v>36</v>
       </c>
@@ -5605,7 +5606,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="172" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A172" t="s">
         <v>31</v>
       </c>
@@ -5634,7 +5635,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="173" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A173" t="s">
         <v>14</v>
       </c>
@@ -5663,7 +5664,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="174" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A174" t="s">
         <v>152</v>
       </c>
@@ -5689,7 +5690,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="175" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A175" t="s">
         <v>116</v>
       </c>
@@ -5712,7 +5713,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="176" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A176" t="s">
         <v>118</v>
       </c>
@@ -5732,7 +5733,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="177" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A177" t="s">
         <v>114</v>
       </c>
@@ -5752,7 +5753,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="178" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A178" t="s">
         <v>62</v>
       </c>
@@ -5781,7 +5782,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="179" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A179" t="s">
         <v>28</v>
       </c>
@@ -5804,7 +5805,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="180" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A180" t="s">
         <v>24</v>
       </c>
@@ -5836,7 +5837,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="181" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A181" t="s">
         <v>110</v>
       </c>
@@ -5871,7 +5872,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="182" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A182" t="s">
         <v>66</v>
       </c>
@@ -5906,7 +5907,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="183" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A183" t="s">
         <v>101</v>
       </c>
@@ -5935,7 +5936,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="184" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A184" t="s">
         <v>139</v>
       </c>
@@ -5955,7 +5956,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="185" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A185" t="s">
         <v>76</v>
       </c>
@@ -5990,7 +5991,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="186" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A186" t="s">
         <v>23</v>
       </c>
@@ -6019,7 +6020,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="187" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A187" t="s">
         <v>48</v>
       </c>
@@ -6045,7 +6046,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="188" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A188" t="s">
         <v>62</v>
       </c>
@@ -6071,7 +6072,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="189" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A189" t="s">
         <v>49</v>
       </c>
@@ -6103,7 +6104,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="190" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A190" t="s">
         <v>84</v>
       </c>
@@ -6135,7 +6136,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="191" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A191" t="s">
         <v>73</v>
       </c>
@@ -6158,7 +6159,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="192" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A192" t="s">
         <v>159</v>
       </c>
@@ -6181,7 +6182,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="193" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A193" t="s">
         <v>11</v>
       </c>
@@ -6204,7 +6205,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="194" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A194" t="s">
         <v>66</v>
       </c>
@@ -6233,7 +6234,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="195" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A195" t="s">
         <v>54</v>
       </c>
@@ -6268,7 +6269,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="196" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A196" t="s">
         <v>121</v>
       </c>
@@ -6291,7 +6292,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="197" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A197" t="s">
         <v>26</v>
       </c>
@@ -6323,7 +6324,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="198" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A198" t="s">
         <v>28</v>
       </c>
@@ -6343,7 +6344,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="199" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A199" t="s">
         <v>14</v>
       </c>
@@ -6363,7 +6364,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="200" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A200" t="s">
         <v>47</v>
       </c>
@@ -6398,7 +6399,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="201" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A201" t="s">
         <v>124</v>
       </c>
@@ -6424,7 +6425,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="202" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A202" t="s">
         <v>118</v>
       </c>
@@ -6456,7 +6457,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="203" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A203" t="s">
         <v>64</v>
       </c>
@@ -6476,7 +6477,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="204" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A204" t="s">
         <v>63</v>
       </c>
@@ -6511,7 +6512,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="205" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A205" t="s">
         <v>41</v>
       </c>
@@ -6537,7 +6538,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="206" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A206" t="s">
         <v>127</v>
       </c>
@@ -6572,7 +6573,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="207" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A207" t="s">
         <v>19</v>
       </c>
@@ -6604,7 +6605,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="208" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A208" t="s">
         <v>69</v>
       </c>
@@ -6624,7 +6625,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="209" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A209" t="s">
         <v>34</v>
       </c>
@@ -6653,7 +6654,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="210" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A210" t="s">
         <v>16</v>
       </c>
@@ -6673,7 +6674,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="211" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A211" t="s">
         <v>24</v>
       </c>
@@ -6699,7 +6700,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="212" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A212" t="s">
         <v>28</v>
       </c>
@@ -6722,7 +6723,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="213" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A213" t="s">
         <v>132</v>
       </c>
@@ -6742,7 +6743,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="214" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A214" t="s">
         <v>66</v>
       </c>
@@ -6777,7 +6778,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="215" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A215" t="s">
         <v>48</v>
       </c>
@@ -6803,7 +6804,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="216" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A216" t="s">
         <v>146</v>
       </c>
@@ -6832,7 +6833,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="217" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A217" t="s">
         <v>64</v>
       </c>
@@ -6861,7 +6862,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="218" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A218" t="s">
         <v>19</v>
       </c>
@@ -6890,7 +6891,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="219" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A219" t="s">
         <v>74</v>
       </c>
@@ -6916,7 +6917,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="220" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A220" t="s">
         <v>55</v>
       </c>
@@ -6945,7 +6946,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="221" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A221" t="s">
         <v>66</v>
       </c>
@@ -6980,7 +6981,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="222" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A222" t="s">
         <v>101</v>
       </c>
@@ -7009,7 +7010,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="223" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A223" t="s">
         <v>32</v>
       </c>
@@ -7032,7 +7033,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="224" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A224" t="s">
         <v>117</v>
       </c>
@@ -7064,7 +7065,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="225" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A225" t="s">
         <v>12</v>
       </c>
@@ -7084,7 +7085,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="226" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A226" t="s">
         <v>71</v>
       </c>
@@ -7107,7 +7108,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="227" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A227" t="s">
         <v>54</v>
       </c>
@@ -7127,7 +7128,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="228" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A228" t="s">
         <v>132</v>
       </c>
@@ -7147,7 +7148,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="229" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A229" t="s">
         <v>88</v>
       </c>
@@ -7182,7 +7183,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="230" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A230" t="s">
         <v>50</v>
       </c>
@@ -7217,7 +7218,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="231" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A231" t="s">
         <v>146</v>
       </c>
@@ -7249,7 +7250,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="232" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A232" t="s">
         <v>12</v>
       </c>
@@ -7269,7 +7270,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="233" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A233" t="s">
         <v>156</v>
       </c>
@@ -7301,7 +7302,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="234" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A234" t="s">
         <v>100</v>
       </c>
@@ -7321,7 +7322,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="235" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A235" t="s">
         <v>42</v>
       </c>
@@ -7347,7 +7348,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="236" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A236" t="s">
         <v>131</v>
       </c>
@@ -7370,7 +7371,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="237" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A237" t="s">
         <v>56</v>
       </c>
@@ -7402,7 +7403,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="238" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A238" t="s">
         <v>50</v>
       </c>
@@ -7434,7 +7435,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="239" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A239" t="s">
         <v>142</v>
       </c>
@@ -7460,7 +7461,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="240" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A240" t="s">
         <v>75</v>
       </c>
@@ -7495,7 +7496,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="241" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A241" t="s">
         <v>41</v>
       </c>
@@ -7521,7 +7522,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="242" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A242" t="s">
         <v>97</v>
       </c>
@@ -7553,7 +7554,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="243" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A243" t="s">
         <v>14</v>
       </c>
@@ -7585,7 +7586,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="244" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A244" t="s">
         <v>71</v>
       </c>
@@ -7605,7 +7606,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="245" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A245" t="s">
         <v>128</v>
       </c>
@@ -7625,7 +7626,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="246" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A246" t="s">
         <v>34</v>
       </c>
@@ -7645,7 +7646,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="247" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A247" t="s">
         <v>28</v>
       </c>
@@ -7665,7 +7666,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="248" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A248" t="s">
         <v>31</v>
       </c>
@@ -7697,7 +7698,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="249" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="249" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A249" t="s">
         <v>157</v>
       </c>
@@ -7732,7 +7733,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="250" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="250" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A250" t="s">
         <v>21</v>
       </c>
@@ -7752,7 +7753,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="251" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="251" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A251" t="s">
         <v>153</v>
       </c>
@@ -7781,7 +7782,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="252" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="252" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A252" t="s">
         <v>31</v>
       </c>
@@ -7816,7 +7817,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="253" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A253" t="s">
         <v>107</v>
       </c>
@@ -7845,7 +7846,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="254" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="254" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A254" t="s">
         <v>76</v>
       </c>
@@ -7865,7 +7866,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="255" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="255" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A255" t="s">
         <v>58</v>
       </c>
@@ -7900,7 +7901,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="256" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="256" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A256" t="s">
         <v>36</v>
       </c>
@@ -7926,7 +7927,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="257" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="257" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A257" t="s">
         <v>144</v>
       </c>
@@ -7961,7 +7962,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="258" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="258" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A258" t="s">
         <v>110</v>
       </c>
@@ -7993,7 +7994,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="259" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="259" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A259" t="s">
         <v>118</v>
       </c>
@@ -8016,7 +8017,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="260" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="260" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A260" t="s">
         <v>28</v>
       </c>
@@ -8036,7 +8037,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="261" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="261" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A261" t="s">
         <v>151</v>
       </c>
@@ -8059,7 +8060,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="262" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="262" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A262" t="s">
         <v>12</v>
       </c>
@@ -8079,7 +8080,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="263" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="263" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A263" t="s">
         <v>154</v>
       </c>
@@ -8108,7 +8109,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="264" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="264" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A264" t="s">
         <v>69</v>
       </c>
@@ -8134,7 +8135,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="265" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="265" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A265" t="s">
         <v>114</v>
       </c>
@@ -8166,7 +8167,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="266" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="266" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A266" t="s">
         <v>106</v>
       </c>
@@ -8186,7 +8187,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="267" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="267" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A267" t="s">
         <v>102</v>
       </c>
@@ -8206,7 +8207,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="268" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="268" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A268" t="s">
         <v>43</v>
       </c>
@@ -8238,7 +8239,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="269" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="269" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A269" t="s">
         <v>58</v>
       </c>
@@ -8270,7 +8271,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="270" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="270" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A270" t="s">
         <v>151</v>
       </c>
@@ -8299,7 +8300,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="271" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="271" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A271" t="s">
         <v>11</v>
       </c>
@@ -8331,7 +8332,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="272" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="272" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A272" t="s">
         <v>50</v>
       </c>
@@ -8357,7 +8358,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="273" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="273" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A273" t="s">
         <v>69</v>
       </c>
@@ -8386,7 +8387,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="274" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="274" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A274" t="s">
         <v>18</v>
       </c>
@@ -8406,7 +8407,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="275" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="275" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A275" t="s">
         <v>100</v>
       </c>
@@ -8435,7 +8436,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="276" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="276" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A276" t="s">
         <v>118</v>
       </c>
@@ -8458,7 +8459,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="277" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="277" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A277" t="s">
         <v>46</v>
       </c>
@@ -8487,7 +8488,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="278" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="278" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A278" t="s">
         <v>12</v>
       </c>
@@ -8510,7 +8511,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="279" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="279" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A279" t="s">
         <v>41</v>
       </c>
@@ -8533,7 +8534,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="280" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="280" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A280" t="s">
         <v>19</v>
       </c>
@@ -8556,7 +8557,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="281" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="281" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A281" t="s">
         <v>28</v>
       </c>
@@ -8591,7 +8592,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="282" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="282" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A282" t="s">
         <v>40</v>
       </c>
@@ -8623,7 +8624,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="283" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="283" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A283" t="s">
         <v>25</v>
       </c>
@@ -8643,7 +8644,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="284" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="284" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A284" t="s">
         <v>142</v>
       </c>
@@ -8666,7 +8667,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="285" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="285" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A285" t="s">
         <v>150</v>
       </c>
@@ -8689,7 +8690,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="286" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="286" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A286" t="s">
         <v>82</v>
       </c>
@@ -8718,7 +8719,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="287" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="287" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A287" t="s">
         <v>50</v>
       </c>
@@ -8738,7 +8739,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="288" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="288" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A288" t="s">
         <v>14</v>
       </c>
@@ -8770,7 +8771,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="289" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="289" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A289" t="s">
         <v>36</v>
       </c>
@@ -8790,7 +8791,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="290" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="290" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A290" t="s">
         <v>155</v>
       </c>
@@ -8816,7 +8817,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="291" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="291" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A291" t="s">
         <v>32</v>
       </c>
@@ -8836,7 +8837,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="292" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="292" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A292" t="s">
         <v>13</v>
       </c>
@@ -8865,7 +8866,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="293" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="293" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A293" t="s">
         <v>14</v>
       </c>
@@ -8900,7 +8901,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="294" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="294" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A294" t="s">
         <v>71</v>
       </c>
@@ -8923,7 +8924,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="295" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="295" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A295" t="s">
         <v>20</v>
       </c>
@@ -8958,7 +8959,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="296" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="296" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A296" t="s">
         <v>13</v>
       </c>
@@ -8981,7 +8982,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="297" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="297" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A297" t="s">
         <v>12</v>
       </c>
@@ -9004,7 +9005,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="298" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="298" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A298" t="s">
         <v>110</v>
       </c>
@@ -9030,7 +9031,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="299" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="299" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A299" t="s">
         <v>32</v>
       </c>
@@ -9053,7 +9054,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="300" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="300" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A300" t="s">
         <v>96</v>
       </c>
@@ -9088,7 +9089,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="301" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="301" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A301" t="s">
         <v>11</v>
       </c>
@@ -9111,7 +9112,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="302" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="302" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A302" t="s">
         <v>45</v>
       </c>
@@ -9137,7 +9138,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="303" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="303" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A303" t="s">
         <v>84</v>
       </c>
@@ -9163,7 +9164,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="304" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="304" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A304" t="s">
         <v>57</v>
       </c>
@@ -9183,7 +9184,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="305" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="305" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A305" t="s">
         <v>116</v>
       </c>
@@ -9212,7 +9213,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="306" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="306" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A306" t="s">
         <v>68</v>
       </c>
@@ -9238,7 +9239,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="307" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="307" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A307" t="s">
         <v>140</v>
       </c>
@@ -9258,7 +9259,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="308" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="308" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A308" t="s">
         <v>68</v>
       </c>
@@ -9284,7 +9285,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="309" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="309" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A309" t="s">
         <v>92</v>
       </c>
@@ -9310,7 +9311,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="310" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="310" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A310" t="s">
         <v>46</v>
       </c>
@@ -9330,7 +9331,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="311" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="311" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A311" t="s">
         <v>37</v>
       </c>
@@ -9359,7 +9360,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="312" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="312" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A312" t="s">
         <v>144</v>
       </c>
@@ -9391,7 +9392,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="313" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="313" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A313" t="s">
         <v>39</v>
       </c>
@@ -9426,7 +9427,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="314" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="314" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A314" t="s">
         <v>81</v>
       </c>
@@ -9449,7 +9450,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="315" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="315" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A315" t="s">
         <v>100</v>
       </c>
@@ -9469,7 +9470,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="316" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="316" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A316" t="s">
         <v>135</v>
       </c>
@@ -9501,7 +9502,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="317" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="317" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A317" t="s">
         <v>118</v>
       </c>
@@ -9524,7 +9525,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="318" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="318" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A318" t="s">
         <v>114</v>
       </c>
@@ -9544,7 +9545,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="319" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="319" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A319" t="s">
         <v>152</v>
       </c>
@@ -9579,7 +9580,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="320" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="320" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A320" t="s">
         <v>36</v>
       </c>
@@ -9611,7 +9612,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="321" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="321" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A321" t="s">
         <v>12</v>
       </c>
@@ -9640,7 +9641,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="322" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="322" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A322" t="s">
         <v>147</v>
       </c>
@@ -9660,7 +9661,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="323" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="323" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A323" t="s">
         <v>40</v>
       </c>
@@ -9692,7 +9693,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="324" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="324" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A324" t="s">
         <v>61</v>
       </c>
@@ -9712,7 +9713,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="325" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="325" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A325" t="s">
         <v>39</v>
       </c>
@@ -9741,7 +9742,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="326" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="326" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A326" t="s">
         <v>28</v>
       </c>
@@ -9764,7 +9765,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="327" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="327" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A327" t="s">
         <v>36</v>
       </c>
@@ -9787,7 +9788,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="328" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="328" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A328" t="s">
         <v>114</v>
       </c>
@@ -9813,7 +9814,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="329" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="329" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A329" t="s">
         <v>49</v>
       </c>
@@ -9842,7 +9843,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="330" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="330" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A330" t="s">
         <v>144</v>
       </c>
@@ -9874,7 +9875,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="331" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="331" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A331" t="s">
         <v>81</v>
       </c>
@@ -9909,7 +9910,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="332" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="332" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A332" t="s">
         <v>48</v>
       </c>
@@ -9944,7 +9945,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="333" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="333" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A333" t="s">
         <v>50</v>
       </c>
@@ -9979,7 +9980,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="334" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="334" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A334" t="s">
         <v>139</v>
       </c>
@@ -10014,7 +10015,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="335" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="335" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A335" t="s">
         <v>144</v>
       </c>
@@ -10043,7 +10044,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="336" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="336" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A336" t="s">
         <v>28</v>
       </c>
@@ -10072,7 +10073,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="337" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="337" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A337" t="s">
         <v>69</v>
       </c>
@@ -10101,7 +10102,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="338" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="338" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A338" t="s">
         <v>13</v>
       </c>
@@ -10133,7 +10134,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="339" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="339" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A339" t="s">
         <v>97</v>
       </c>
@@ -10153,7 +10154,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="340" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="340" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A340" t="s">
         <v>88</v>
       </c>
@@ -10182,7 +10183,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="341" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="341" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A341" t="s">
         <v>159</v>
       </c>
@@ -10211,7 +10212,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="342" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="342" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A342" t="s">
         <v>151</v>
       </c>
@@ -10246,7 +10247,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="343" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="343" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A343" t="s">
         <v>29</v>
       </c>
@@ -10281,7 +10282,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="344" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="344" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A344" t="s">
         <v>149</v>
       </c>
@@ -10301,7 +10302,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="345" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="345" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A345" t="s">
         <v>49</v>
       </c>
@@ -10330,7 +10331,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="346" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="346" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A346" t="s">
         <v>94</v>
       </c>
@@ -10353,7 +10354,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="347" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="347" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A347" t="s">
         <v>142</v>
       </c>
@@ -10385,7 +10386,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="348" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="348" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A348" t="s">
         <v>20</v>
       </c>
@@ -10417,7 +10418,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="349" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="349" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A349" t="s">
         <v>103</v>
       </c>
@@ -10449,7 +10450,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="350" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="350" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A350" t="s">
         <v>66</v>
       </c>
@@ -10469,7 +10470,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="351" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="351" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A351" t="s">
         <v>142</v>
       </c>
@@ -10501,7 +10502,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="352" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="352" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A352" t="s">
         <v>111</v>
       </c>
@@ -10530,7 +10531,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="353" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="353" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A353" t="s">
         <v>52</v>
       </c>
@@ -10565,7 +10566,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="354" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="354" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A354" t="s">
         <v>144</v>
       </c>
@@ -10597,7 +10598,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="355" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="355" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A355" t="s">
         <v>96</v>
       </c>
@@ -10620,7 +10621,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="356" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="356" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A356" t="s">
         <v>116</v>
       </c>
@@ -10643,7 +10644,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="357" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="357" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A357" t="s">
         <v>30</v>
       </c>
@@ -10669,7 +10670,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="358" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="358" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A358" t="s">
         <v>146</v>
       </c>
@@ -10704,7 +10705,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="359" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="359" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A359" t="s">
         <v>148</v>
       </c>
@@ -10739,7 +10740,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="360" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="360" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A360" t="s">
         <v>76</v>
       </c>
@@ -10771,7 +10772,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="361" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="361" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A361" t="s">
         <v>50</v>
       </c>
@@ -10800,7 +10801,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="362" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="362" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A362" t="s">
         <v>69</v>
       </c>
@@ -10826,7 +10827,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="363" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="363" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A363" t="s">
         <v>25</v>
       </c>
@@ -10855,7 +10856,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="364" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="364" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A364" t="s">
         <v>11</v>
       </c>
@@ -10878,7 +10879,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="365" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="365" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A365" t="s">
         <v>107</v>
       </c>
@@ -10901,7 +10902,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="366" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="366" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A366" t="s">
         <v>135</v>
       </c>
@@ -10921,7 +10922,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="367" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="367" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A367" t="s">
         <v>51</v>
       </c>
@@ -10956,7 +10957,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="368" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="368" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A368" t="s">
         <v>13</v>
       </c>
@@ -10985,7 +10986,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="369" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="369" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A369" t="s">
         <v>159</v>
       </c>
@@ -11017,7 +11018,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="370" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="370" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A370" t="s">
         <v>57</v>
       </c>
@@ -11040,7 +11041,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="371" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="371" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A371" t="s">
         <v>12</v>
       </c>
@@ -11072,7 +11073,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="372" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="372" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A372" t="s">
         <v>110</v>
       </c>
@@ -11095,7 +11096,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="373" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="373" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A373" t="s">
         <v>49</v>
       </c>
@@ -11118,7 +11119,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="374" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="374" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A374" t="s">
         <v>49</v>
       </c>
@@ -11138,7 +11139,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="375" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="375" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A375" t="s">
         <v>28</v>
       </c>
@@ -11167,7 +11168,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="376" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="376" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A376" t="s">
         <v>69</v>
       </c>
@@ -11199,7 +11200,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="377" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="377" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A377" t="s">
         <v>50</v>
       </c>
@@ -11225,7 +11226,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="378" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="378" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A378" t="s">
         <v>38</v>
       </c>
@@ -11260,7 +11261,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="379" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="379" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A379" t="s">
         <v>15</v>
       </c>
@@ -11286,7 +11287,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="380" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="380" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A380" t="s">
         <v>155</v>
       </c>
@@ -11315,7 +11316,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="381" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="381" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A381" t="s">
         <v>64</v>
       </c>
@@ -11341,7 +11342,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="382" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="382" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A382" t="s">
         <v>48</v>
       </c>
@@ -11370,7 +11371,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="383" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="383" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A383" t="s">
         <v>143</v>
       </c>
@@ -11396,7 +11397,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="384" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="384" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A384" t="s">
         <v>122</v>
       </c>
@@ -11425,7 +11426,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="385" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="385" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A385" t="s">
         <v>19</v>
       </c>
@@ -11445,7 +11446,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="386" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="386" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A386" t="s">
         <v>73</v>
       </c>
@@ -11471,7 +11472,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="387" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="387" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A387" t="s">
         <v>28</v>
       </c>
@@ -11500,7 +11501,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="388" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="388" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A388" t="s">
         <v>12</v>
       </c>
@@ -11526,7 +11527,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="389" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="389" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A389" t="s">
         <v>120</v>
       </c>
@@ -11552,7 +11553,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="390" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="390" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A390" t="s">
         <v>118</v>
       </c>
@@ -11581,7 +11582,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="391" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="391" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A391" t="s">
         <v>87</v>
       </c>
@@ -11616,7 +11617,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="392" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="392" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A392" t="s">
         <v>14</v>
       </c>
@@ -11636,7 +11637,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="393" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="393" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A393" t="s">
         <v>63</v>
       </c>
@@ -11656,7 +11657,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="394" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="394" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A394" t="s">
         <v>62</v>
       </c>
@@ -11682,7 +11683,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="395" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="395" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A395" t="s">
         <v>28</v>
       </c>
@@ -11702,7 +11703,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="396" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="396" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A396" t="s">
         <v>75</v>
       </c>
@@ -11722,7 +11723,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="397" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="397" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A397" t="s">
         <v>57</v>
       </c>
@@ -11754,7 +11755,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="398" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="398" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A398" t="s">
         <v>49</v>
       </c>
@@ -11786,7 +11787,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="399" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="399" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A399" t="s">
         <v>96</v>
       </c>
@@ -11821,7 +11822,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="400" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="400" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A400" t="s">
         <v>144</v>
       </c>
@@ -11844,7 +11845,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="401" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="401" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A401" t="s">
         <v>49</v>
       </c>
@@ -11867,7 +11868,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="402" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="402" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A402" t="s">
         <v>89</v>
       </c>
@@ -11887,7 +11888,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="403" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="403" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A403" t="s">
         <v>50</v>
       </c>
@@ -11907,7 +11908,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="404" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="404" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A404" t="s">
         <v>68</v>
       </c>
@@ -11942,7 +11943,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="405" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="405" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A405" t="s">
         <v>73</v>
       </c>
@@ -11974,7 +11975,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="406" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="406" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A406" t="s">
         <v>89</v>
       </c>
@@ -12009,7 +12010,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="407" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="407" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A407" t="s">
         <v>68</v>
       </c>
@@ -12041,7 +12042,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="408" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="408" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A408" t="s">
         <v>155</v>
       </c>
@@ -12064,7 +12065,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="409" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="409" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A409" t="s">
         <v>142</v>
       </c>
@@ -12087,7 +12088,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="410" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="410" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A410" t="s">
         <v>86</v>
       </c>
@@ -12122,7 +12123,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="411" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="411" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A411" t="s">
         <v>88</v>
       </c>
@@ -12148,7 +12149,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="412" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="412" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A412" t="s">
         <v>75</v>
       </c>
@@ -12180,7 +12181,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="413" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="413" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A413" t="s">
         <v>54</v>
       </c>
@@ -12200,7 +12201,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="414" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="414" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A414" t="s">
         <v>62</v>
       </c>
@@ -12226,7 +12227,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="415" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="415" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A415" t="s">
         <v>109</v>
       </c>
@@ -12249,7 +12250,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="416" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="416" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A416" t="s">
         <v>33</v>
       </c>
@@ -12269,7 +12270,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="417" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="417" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A417" t="s">
         <v>110</v>
       </c>
@@ -12292,7 +12293,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="418" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="418" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A418" t="s">
         <v>11</v>
       </c>
@@ -12324,7 +12325,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="419" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="419" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A419" t="s">
         <v>89</v>
       </c>
@@ -12353,7 +12354,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="420" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="420" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A420" t="s">
         <v>69</v>
       </c>
@@ -12388,7 +12389,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="421" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="421" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A421" t="s">
         <v>63</v>
       </c>
@@ -12408,7 +12409,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="422" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="422" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A422" t="s">
         <v>20</v>
       </c>
@@ -12443,7 +12444,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="423" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="423" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A423" t="s">
         <v>24</v>
       </c>
@@ -12463,7 +12464,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="424" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="424" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A424" t="s">
         <v>71</v>
       </c>
@@ -12492,7 +12493,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="425" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="425" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A425" t="s">
         <v>146</v>
       </c>
@@ -12518,7 +12519,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="426" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="426" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A426" t="s">
         <v>56</v>
       </c>
@@ -12550,7 +12551,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="427" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="427" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A427" t="s">
         <v>73</v>
       </c>
@@ -12582,7 +12583,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="428" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="428" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A428" t="s">
         <v>58</v>
       </c>
@@ -12611,7 +12612,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="429" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="429" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A429" t="s">
         <v>76</v>
       </c>
@@ -12637,7 +12638,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="430" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="430" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A430" t="s">
         <v>61</v>
       </c>
@@ -12660,7 +12661,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="431" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="431" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A431" t="s">
         <v>11</v>
       </c>
@@ -12689,7 +12690,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="432" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="432" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A432" t="s">
         <v>20</v>
       </c>
@@ -12709,7 +12710,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="433" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="433" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A433" t="s">
         <v>142</v>
       </c>
@@ -12732,7 +12733,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="434" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="434" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A434" t="s">
         <v>92</v>
       </c>
@@ -12752,7 +12753,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="435" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="435" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A435" t="s">
         <v>103</v>
       </c>
@@ -12784,7 +12785,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="436" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="436" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A436" t="s">
         <v>28</v>
       </c>
@@ -12804,7 +12805,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="437" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="437" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A437" t="s">
         <v>41</v>
       </c>
@@ -12833,7 +12834,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="438" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="438" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A438" t="s">
         <v>131</v>
       </c>
@@ -12853,7 +12854,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="439" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="439" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A439" t="s">
         <v>73</v>
       </c>
@@ -12876,7 +12877,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="440" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="440" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A440" t="s">
         <v>66</v>
       </c>
@@ -12899,7 +12900,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="441" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="441" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A441" t="s">
         <v>101</v>
       </c>
@@ -12925,7 +12926,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="442" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="442" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A442" t="s">
         <v>11</v>
       </c>
@@ -12957,7 +12958,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="443" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="443" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A443" t="s">
         <v>97</v>
       </c>
@@ -12986,7 +12987,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="444" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="444" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A444" t="s">
         <v>107</v>
       </c>
@@ -13018,7 +13019,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="445" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="445" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A445" t="s">
         <v>157</v>
       </c>
@@ -13038,7 +13039,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="446" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="446" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A446" t="s">
         <v>97</v>
       </c>
@@ -13067,7 +13068,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="447" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="447" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A447" t="s">
         <v>28</v>
       </c>
@@ -13099,7 +13100,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="448" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="448" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A448" t="s">
         <v>60</v>
       </c>
@@ -13134,7 +13135,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="449" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="449" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A449" t="s">
         <v>127</v>
       </c>
@@ -13154,7 +13155,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="450" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="450" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A450" t="s">
         <v>37</v>
       </c>
@@ -13183,7 +13184,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="451" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="451" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A451" t="s">
         <v>84</v>
       </c>
@@ -13206,7 +13207,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="452" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="452" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A452" t="s">
         <v>13</v>
       </c>
@@ -13226,7 +13227,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="453" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="453" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A453" t="s">
         <v>136</v>
       </c>
@@ -13261,7 +13262,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="454" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="454" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A454" t="s">
         <v>74</v>
       </c>
@@ -13290,7 +13291,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="455" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="455" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A455" t="s">
         <v>84</v>
       </c>
@@ -13319,7 +13320,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="456" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="456" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A456" t="s">
         <v>19</v>
       </c>
@@ -13342,7 +13343,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="457" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="457" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A457" t="s">
         <v>61</v>
       </c>
@@ -13377,7 +13378,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="458" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="458" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A458" t="s">
         <v>12</v>
       </c>
@@ -13406,7 +13407,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="459" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="459" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A459" t="s">
         <v>154</v>
       </c>
@@ -13429,7 +13430,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="460" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="460" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A460" t="s">
         <v>31</v>
       </c>
@@ -13449,7 +13450,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="461" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="461" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A461" t="s">
         <v>41</v>
       </c>
@@ -13475,7 +13476,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="462" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="462" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A462" t="s">
         <v>89</v>
       </c>
@@ -13498,7 +13499,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="463" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="463" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A463" t="s">
         <v>89</v>
       </c>
@@ -13524,7 +13525,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="464" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="464" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A464" t="s">
         <v>140</v>
       </c>
@@ -13544,7 +13545,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="465" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="465" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A465" t="s">
         <v>50</v>
       </c>
@@ -13570,7 +13571,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="466" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="466" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A466" t="s">
         <v>62</v>
       </c>
@@ -13602,7 +13603,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="467" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="467" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A467" t="s">
         <v>87</v>
       </c>
@@ -13622,7 +13623,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="468" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="468" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A468" t="s">
         <v>11</v>
       </c>
@@ -13648,7 +13649,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="469" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="469" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A469" t="s">
         <v>142</v>
       </c>
@@ -13680,7 +13681,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="470" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="470" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A470" t="s">
         <v>155</v>
       </c>
@@ -13709,7 +13710,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="471" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="471" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A471" t="s">
         <v>149</v>
       </c>
@@ -13738,7 +13739,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="472" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="472" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A472" t="s">
         <v>125</v>
       </c>
@@ -13767,7 +13768,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="473" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="473" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A473" t="s">
         <v>41</v>
       </c>
@@ -13787,7 +13788,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="474" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="474" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A474" t="s">
         <v>99</v>
       </c>
@@ -13822,7 +13823,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="475" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="475" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A475" t="s">
         <v>63</v>
       </c>
@@ -13857,7 +13858,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="476" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="476" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A476" t="s">
         <v>149</v>
       </c>
@@ -13883,7 +13884,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="477" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="477" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A477" t="s">
         <v>49</v>
       </c>
@@ -13909,7 +13910,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="478" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="478" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A478" t="s">
         <v>91</v>
       </c>
@@ -13938,7 +13939,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="479" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="479" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A479" t="s">
         <v>47</v>
       </c>
@@ -13964,7 +13965,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="480" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="480" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A480" t="s">
         <v>28</v>
       </c>
@@ -13987,7 +13988,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="481" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="481" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A481" t="s">
         <v>148</v>
       </c>
@@ -14013,7 +14014,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="482" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="482" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A482" t="s">
         <v>132</v>
       </c>
@@ -14045,7 +14046,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="483" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="483" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A483" t="s">
         <v>28</v>
       </c>
@@ -14077,7 +14078,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="484" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="484" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A484" t="s">
         <v>78</v>
       </c>
@@ -14112,7 +14113,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="485" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="485" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A485" t="s">
         <v>126</v>
       </c>
@@ -14147,7 +14148,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="486" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="486" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A486" t="s">
         <v>36</v>
       </c>
@@ -14170,7 +14171,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="487" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="487" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A487" t="s">
         <v>150</v>
       </c>
@@ -14205,7 +14206,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="488" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="488" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A488" t="s">
         <v>75</v>
       </c>
@@ -14237,7 +14238,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="489" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="489" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A489" t="s">
         <v>118</v>
       </c>
@@ -14269,7 +14270,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="490" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="490" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A490" t="s">
         <v>89</v>
       </c>
@@ -14289,7 +14290,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="491" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="491" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A491" t="s">
         <v>36</v>
       </c>
@@ -14315,7 +14316,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="492" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="492" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A492" t="s">
         <v>12</v>
       </c>
@@ -14335,7 +14336,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="493" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="493" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A493" t="s">
         <v>33</v>
       </c>
@@ -14355,7 +14356,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="494" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="494" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A494" t="s">
         <v>24</v>
       </c>
@@ -14387,7 +14388,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="495" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="495" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A495" t="s">
         <v>30</v>
       </c>
@@ -14419,7 +14420,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="496" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="496" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A496" t="s">
         <v>143</v>
       </c>
@@ -14454,7 +14455,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="497" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="497" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A497" t="s">
         <v>14</v>
       </c>
@@ -14486,7 +14487,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="498" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="498" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A498" t="s">
         <v>70</v>
       </c>
@@ -14515,7 +14516,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="499" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="499" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A499" t="s">
         <v>25</v>
       </c>
@@ -14538,7 +14539,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="500" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="500" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A500" t="s">
         <v>155</v>
       </c>
@@ -14558,7 +14559,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="501" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="501" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A501" t="s">
         <v>50</v>
       </c>

</xml_diff>